<commit_message>
Updated production curriculum subjects list in Excel sheet
</commit_message>
<xml_diff>
--- a/subjects.xlsx
+++ b/subjects.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,6 +548,138 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HINDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ENGLISH</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MATHS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ART</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>GK</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>URDU</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>SCIENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SOCIAL SCIENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Fourth</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ATTANDANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>FIRST</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>HINDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>FIRST</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ENGLISH</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>